<commit_message>
Feb 06 2024 changes - TMTT0038660
</commit_message>
<xml_diff>
--- a/TestData/TMTT0013748_TMTT0013750_TMTT0013751_TMTT0013753_VerifyNewTitleRateSheetAvailability_CalculatedAmountOnTimeRecordManagerAfterAddingRateSheet.xlsx
+++ b/TestData/TMTT0013748_TMTT0013750_TMTT0013751_TMTT0013753_VerifyNewTitleRateSheetAvailability_CalculatedAmountOnTimeRecordManagerAfterAddingRateSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0B539C-773B-47C1-ACD7-91CD0651C2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA0D63F0-4800-43A9-8E83-A62E0E58A7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="763" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="763" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="8" r:id="rId1"/>

</xml_diff>